<commit_message>
fix(import): scope the currency validation back to the Currency column
Inserting ExchangeRate at J widened the existing currency list-validation
from I2:I1000 to I2:J1000. With errorStyle="stop" that made Excel reject
any decimal typed into ExchangeRate unless it happened to read PHP or USD,
so the column the previous wave added to unblock USD imports was itself
unreachable. Narrows the currency validation back to I2:I1000 and gives
J2:J1000 its own validation (decimal, greater than 0).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/AssetDesk.Web/wwwroot/templates/Asset_Upload_Template.xlsx
+++ b/src/AssetDesk.Web/wwwroot/templates/Asset_Upload_Template.xlsx
@@ -19,25 +19,25 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
-    <x:t xml:space="preserve">  • Currency: PHP, USD</x:t>
+    <x:t xml:space="preserve">  • Currency defaults to PHP if left blank.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">  • ExchangeRate is pesos per 1 unit of Currency — required for any currency other than PHP.</x:t>
   </x:si>
   <x:si>
-    <x:t>USD</x:t>
+    <x:t xml:space="preserve">  • Totals are reported in pesos; each asset keeps the price and currency you enter here.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">  • Currency: PHP, USD</x:t>
   </x:si>
   <x:si>
     <x:t>ExchangeRate</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">  • Currency defaults to PHP if left blank.</x:t>
+    <x:t>PHP</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">  • Totals are reported in pesos; each asset keeps the price and currency you enter here.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PHP</x:t>
+    <x:t>USD</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -667,7 +667,7 @@
     <x:pageSetUpPr/>
   </x:sheetPr>
   <x:dimension ref="A1:A25"/>
-  <x:sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <x:sheetFormatPr baseColWidth="8" defaultColWidth="9.139196" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="110" style="0" customWidth="1"/>
   </x:cols>
@@ -788,7 +788,7 @@
     </x:row>
     <x:row r="19" spans="1:1">
       <x:c r="A19" s="2" t="s">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:1">
@@ -798,7 +798,7 @@
     </x:row>
     <x:row r="21" spans="1:1">
       <x:c r="A21" s="2" t="s">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:1">
@@ -834,7 +834,7 @@
     </x:row>
     <x:row r="27" spans="1:1">
       <x:c r="A27" s="2" t="s">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -853,7 +853,7 @@
     <x:pageSetUpPr/>
   </x:sheetPr>
   <x:dimension ref="A1:O2"/>
-  <x:sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <x:sheetFormatPr baseColWidth="8" defaultColWidth="9.139196" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="22" style="0" customWidth="1"/>
     <x:col min="2" max="3" width="14" style="0" customWidth="1"/>
@@ -917,7 +917,7 @@
         </x:is>
       </x:c>
       <x:c r="J1" s="11" t="s">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K1" s="11" t="inlineStr">
         <x:is>
@@ -1027,7 +1027,7 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="3">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Value must come from the Reference sheet." promptTitle="Pick from list" prompt="Choose a device type" sqref="B2:B1000">
       <x:formula1>=Reference!$A$2:$A$12</x:formula1>
       <x:formula2/>
@@ -1036,8 +1036,12 @@
       <x:formula1>=Reference!$B$2:$B$6</x:formula1>
       <x:formula2/>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Value must come from the Reference sheet." promptTitle="Pick from list" prompt="Choose a currency" sqref="I2:J1000">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Value must come from the Reference sheet." promptTitle="Pick from list" prompt="Choose a currency" sqref="I2:I1000">
       <x:formula1>=Reference!$C$2:$C$3</x:formula1>
+      <x:formula2/>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" errorStyle="stop" operator="greaterThan" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Value must be a number greater than 0." promptTitle="Enter a number" prompt="Enter the exchange rate to PHP" sqref="J2:J1000">
+      <x:formula1>0</x:formula1>
       <x:formula2/>
     </x:dataValidation>
   </x:dataValidations>
@@ -1057,7 +1061,7 @@
     <x:pageSetUpPr/>
   </x:sheetPr>
   <x:dimension ref="A1:C12"/>
-  <x:sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <x:sheetFormatPr baseColWidth="8" defaultColWidth="9.139196" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="2" width="16" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="12" style="0" customWidth="1"/>
@@ -1092,7 +1096,7 @@
         </x:is>
       </x:c>
       <x:c r="C2" s="10" t="s">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
@@ -1107,7 +1111,7 @@
         </x:is>
       </x:c>
       <x:c r="C3" s="10" t="s">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3">

</xml_diff>